<commit_message>
feat(carga): proyectos con historial comercial y tipos de proyecto del negocio
- Plantilla de proyectos v2: cliente por codigo de cliente, unidad y cantidad,
  fase del cliente con avance, y oportunidad con etapa, resultado, motivo,
  porcentaje y fecha de decision historica (ADR-031).
- Validacion previa de reglas de resultado, motivo, transiciones y avance;
  pasos posteriores fallidos quedan como "creada con advertencia".
- Semilla: 16 tipos de proyecto, fases INICIAL y PARALIZADO, etapa
  SIN_CONTACTAR y unidades KM, PZA, ROL, CJS, PAQ, SET y SAC.
- Plantillas regeneradas, documentacion y pruebas unitarias y e2e.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/plantilla-productos.xlsx
+++ b/docs/templates/plantilla-productos.xlsx
@@ -640,7 +640,7 @@
         <v>Versión de plantilla</v>
       </c>
       <c r="B11" s="1" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="str">
@@ -774,6 +774,83 @@
         <v>Varilla</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>KM</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>Kilómetro</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <v>PZA</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <v>Pieza</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <v>ROL</v>
+      </c>
+      <c r="C13" s="1" t="str">
+        <v>Rollo</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B14" s="1" t="str">
+        <v>CJS</v>
+      </c>
+      <c r="C14" s="1" t="str">
+        <v>Caja</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B15" s="1" t="str">
+        <v>PAQ</v>
+      </c>
+      <c r="C15" s="1" t="str">
+        <v>Paquete</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B16" s="1" t="str">
+        <v>SET</v>
+      </c>
+      <c r="C16" s="1" t="str">
+        <v>Juego</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="str">
+        <v>Código de unidad base</v>
+      </c>
+      <c r="B17" s="1" t="str">
+        <v>SAC</v>
+      </c>
+      <c r="C17" s="1" t="str">
+        <v>Saco</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>